<commit_message>
docs: clarify lookahead report implementation conditions
</commit_message>
<xml_diff>
--- a/lookahead_learning/docs/前方注視点_入力と報酬_報告書.xlsx
+++ b/lookahead_learning/docs/前方注視点_入力と報酬_報告書.xlsx
@@ -1291,10 +1291,10 @@
     </r>
   </si>
   <si>
-    <t>この2距離を正規化し、有効フラグとともに既存観測の末尾へ追加する。</t>
-  </si>
-  <si>
-    <t>元の D 要素は保ち、以下の順で3要素を追加する（合計 D+3 要素）。</t>
+    <t>設定に [lookahead] がある場合、2距離の正規化値と有効フラグを既存観測の末尾へ追加する。</t>
+  </si>
+  <si>
+    <t>元の D 要素に次の3要素を追加する（D+3）。[lookahead] がなければ元の D 要素を返す。</t>
   </si>
   <si>
     <t>順序</t>
@@ -1918,7 +1918,7 @@
         <family val="3"/>
         <charset val="128"/>
       </rPr>
-      <t xml:space="preserve"> は報酬重み（pp_weight、0以上）。Δt は1行動ステップの時間 [s]（通常0.1秒）。</t>
+      <t xml:space="preserve"> は報酬重み pp_weight ≥ 0（既定0.0、正値で有効）。Δt は1行動の時間 [s]（通常0.1秒）。</t>
     </r>
   </si>
   <si>
@@ -1970,7 +1970,7 @@
         <family val="3"/>
         <charset val="128"/>
       </rPr>
-      <t xml:space="preserve"> は最大操舵角 [deg]。本環境は 40°、操舵の正方向は左。</t>
+      <t xml:space="preserve"> は最大操舵角 [deg]。車両の max_steering（既定40°）を使う。正方向は左。</t>
     </r>
   </si>
   <si>
@@ -2126,7 +2126,9 @@
   </si>
   <si>
     <t>端点・接線方向・車線数・幅が連続し、接続可能な車線が
-開始車線番号の候補1本だけであることを確認する。</t>
+開始車線番号の候補1本だけであることを確認する。
+既定の許容誤差は、端点距離・幅差 0.001 m、
+接線方向差 0.001 rad。車線数は一致が必要。</t>
   </si>
   <si>
     <t>確認できた中心線を進行方向につなぐ。
@@ -3466,7 +3468,7 @@
       <c r="T8" s="25"/>
       <c r="U8" s="9"/>
     </row>
-    <row r="9" spans="1:21" ht="54" customHeight="1">
+    <row r="9" spans="1:21" ht="72" customHeight="1">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="23" t="s">

</xml_diff>